<commit_message>
docs: log Rex's self-reported contribution hours in tracker
</commit_message>
<xml_diff>
--- a/project_docs/FamilyPulse_Feature_Tracker.xlsx
+++ b/project_docs/FamilyPulse_Feature_Tracker.xlsx
@@ -347,7 +347,7 @@
     <t xml:space="preserve">Firestore wiring for calendar &amp; events (create/edit/delete), validation and error/success UX across auth + event editor, Welcome screen and auth gating, sign-out relocation + confirmation, theme system + Settings screen, Firestore security-rules fix for first-time family joins, Analytics page, Free Time finder screen, Family Groups, expanded roles + parent-rename (with matching security rules), real event categories, nav drawer + Profile screen, CI build-failure email alerts, several bug fixes (dialog crash, family-code race, pre-commit hook).</t>
   </si>
   <si>
-    <t xml:space="preserve">Hours are an example placeholder format — fill in real logged hours.</t>
+    <t xml:space="preserve">Self-reported by Rex (as of Aug 26, 2026): ~200 hours total across research, core app build, Firebase/Storage setup, and CI/CD pipeline work. An estimate, not independently timestamped.</t>
   </si>
   <si>
     <t xml:space="preserve">Jimmy Söderström</t>
@@ -1471,7 +1471,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="6" t="s">
         <v>96</v>
       </c>
@@ -1569,7 +1569,9 @@
       <c r="C5" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="D5" s="10"/>
+      <c r="D5" s="10" t="n">
+        <v>200</v>
+      </c>
       <c r="E5" s="6" t="s">
         <v>108</v>
       </c>
@@ -1625,7 +1627,7 @@
       </c>
       <c r="D10" s="5" t="n">
         <f aca="false">SUM(D5:D8)</f>
-        <v>0</v>
+        <v>200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>